<commit_message>
change suspect upper limit for water temp
</commit_message>
<xml_diff>
--- a/inst/extdata/ExampleMeta.xlsx
+++ b/inst/extdata/ExampleMeta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33FAB42F-B0F4-411D-91EE-9636581D8650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5B3C6D-F195-42B9-A179-840C1AEA32DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36405" yWindow="3270" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -444,21 +444,21 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -525,7 +525,7 @@
         <v>-0.5</v>
       </c>
       <c r="G2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H2">
         <v>2</v>

</xml_diff>

<commit_message>
update roc to match logic in contdataqc
</commit_message>
<xml_diff>
--- a/inst/extdata/ExampleMeta.xlsx
+++ b/inst/extdata/ExampleMeta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5B3C6D-F195-42B9-A179-840C1AEA32DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A22F463-0FCA-4B7C-9EA3-DE12A72B2D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36405" yWindow="3270" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,9 +49,6 @@
     <t>FlatSuspectDelta</t>
   </si>
   <si>
-    <t>RoCStdev</t>
-  </si>
-  <si>
     <t>RoCHours</t>
   </si>
   <si>
@@ -89,6 +86,9 @@
   </si>
   <si>
     <t>GrMaxSuspect</t>
+  </si>
+  <si>
+    <t>RoCN</t>
   </si>
 </sst>
 </file>
@@ -472,16 +472,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -502,18 +502,18 @@
         <v>8</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
       </c>
       <c r="D2">
         <v>-1</v>
@@ -554,10 +554,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>-1</v>
@@ -598,10 +598,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -642,10 +642,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -686,10 +686,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6">
         <v>10</v>
@@ -730,10 +730,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -774,10 +774,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>3</v>

</xml_diff>

<commit_message>
remote site and depth from entire workflow
</commit_message>
<xml_diff>
--- a/inst/extdata/ExampleMeta.xlsx
+++ b/inst/extdata/ExampleMeta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proj\AquaSensR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A22F463-0FCA-4B7C-9EA3-DE12A72B2D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B88ECB-6D53-49D7-9004-354243B7F6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36405" yWindow="3270" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="3120" windowWidth="26910" windowHeight="10770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,17 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
-  <si>
-    <t>Site</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Parameter</t>
   </si>
   <si>
-    <t>Depth</t>
-  </si>
-  <si>
     <t>SpikeFail</t>
   </si>
   <si>
@@ -50,9 +44,6 @@
   </si>
   <si>
     <t>RoCHours</t>
-  </si>
-  <si>
-    <t>sud096</t>
   </si>
   <si>
     <t>Water Temp_C</t>
@@ -441,47 +432,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -496,323 +485,296 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="B2">
+        <v>-1</v>
+      </c>
+      <c r="C2">
+        <v>30</v>
+      </c>
+      <c r="D2">
+        <v>-0.5</v>
+      </c>
+      <c r="E2">
+        <v>28</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>1.5</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
+      <c r="I2">
+        <v>0.01</v>
+      </c>
+      <c r="J2">
+        <v>60</v>
+      </c>
+      <c r="K2">
+        <v>0.01</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
+      <c r="B3">
+        <v>-1</v>
+      </c>
+      <c r="C3">
+        <v>120</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+      <c r="H3">
+        <v>60</v>
+      </c>
+      <c r="I3">
+        <v>0.01</v>
+      </c>
+      <c r="J3">
+        <v>30</v>
+      </c>
+      <c r="K3">
+        <v>0.01</v>
+      </c>
+      <c r="L3">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2">
-        <v>-1</v>
-      </c>
-      <c r="E2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>18</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>60</v>
+      </c>
+      <c r="I4">
+        <v>0.01</v>
+      </c>
+      <c r="J4">
         <v>30</v>
       </c>
-      <c r="F2">
-        <v>-0.5</v>
-      </c>
-      <c r="G2">
-        <v>28</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>1.5</v>
-      </c>
-      <c r="J2">
-        <v>100</v>
-      </c>
-      <c r="K2">
-        <v>0.01</v>
-      </c>
-      <c r="L2">
-        <v>60</v>
-      </c>
-      <c r="M2">
-        <v>0.01</v>
-      </c>
-      <c r="N2">
+      <c r="K4">
+        <v>0.01</v>
+      </c>
+      <c r="L4">
         <v>6</v>
       </c>
-      <c r="O2">
+      <c r="M4">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3">
-        <v>-1</v>
-      </c>
-      <c r="E3">
-        <v>120</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>100</v>
-      </c>
-      <c r="H3">
-        <v>25</v>
-      </c>
-      <c r="I3">
-        <v>10</v>
-      </c>
-      <c r="J3">
-        <v>60</v>
-      </c>
-      <c r="K3">
-        <v>0.01</v>
-      </c>
-      <c r="L3">
-        <v>30</v>
-      </c>
-      <c r="M3">
-        <v>0.01</v>
-      </c>
-      <c r="N3">
-        <v>6</v>
-      </c>
-      <c r="O3">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>18</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>16</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>60</v>
-      </c>
-      <c r="K4">
-        <v>0.01</v>
-      </c>
-      <c r="L4">
-        <v>30</v>
-      </c>
-      <c r="M4">
-        <v>0.01</v>
-      </c>
-      <c r="N4">
-        <v>6</v>
-      </c>
-      <c r="O4">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>1500</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>1200</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>60</v>
+      </c>
+      <c r="I5">
+        <v>0.01</v>
+      </c>
+      <c r="J5">
+        <v>30</v>
+      </c>
+      <c r="K5">
+        <v>0.01</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
+      </c>
+      <c r="M5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="D5">
+      <c r="B6">
         <v>10</v>
       </c>
-      <c r="E5">
+      <c r="C6">
         <v>1500</v>
       </c>
-      <c r="F5">
+      <c r="D6">
         <v>20</v>
       </c>
-      <c r="G5">
+      <c r="E6">
         <v>1200</v>
       </c>
-      <c r="H5">
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <v>50</v>
+      </c>
+      <c r="H6">
+        <v>60</v>
+      </c>
+      <c r="I6">
+        <v>0.01</v>
+      </c>
+      <c r="J6">
+        <v>30</v>
+      </c>
+      <c r="K6">
+        <v>0.01</v>
+      </c>
+      <c r="L6">
+        <v>6</v>
+      </c>
+      <c r="M6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>41</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>37</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>60</v>
+      </c>
+      <c r="I7">
+        <v>0.01</v>
+      </c>
+      <c r="J7">
+        <v>30</v>
+      </c>
+      <c r="K7">
+        <v>0.01</v>
+      </c>
+      <c r="L7">
+        <v>6</v>
+      </c>
+      <c r="M7">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>11</v>
+      </c>
+      <c r="F8">
         <v>10</v>
       </c>
-      <c r="I5">
+      <c r="G8">
         <v>5</v>
       </c>
-      <c r="J5">
+      <c r="H8">
         <v>60</v>
       </c>
-      <c r="K5">
-        <v>0.01</v>
-      </c>
-      <c r="L5">
+      <c r="I8">
+        <v>0.01</v>
+      </c>
+      <c r="J8">
         <v>30</v>
       </c>
-      <c r="M5">
-        <v>0.01</v>
-      </c>
-      <c r="N5">
+      <c r="K8">
+        <v>0.01</v>
+      </c>
+      <c r="L8">
         <v>6</v>
       </c>
-      <c r="O5">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>1500</v>
-      </c>
-      <c r="F6">
-        <v>20</v>
-      </c>
-      <c r="G6">
-        <v>1200</v>
-      </c>
-      <c r="H6">
-        <v>100</v>
-      </c>
-      <c r="I6">
-        <v>50</v>
-      </c>
-      <c r="J6">
-        <v>60</v>
-      </c>
-      <c r="K6">
-        <v>0.01</v>
-      </c>
-      <c r="L6">
-        <v>30</v>
-      </c>
-      <c r="M6">
-        <v>0.01</v>
-      </c>
-      <c r="N6">
-        <v>6</v>
-      </c>
-      <c r="O6">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>41</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="G7">
-        <v>37</v>
-      </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>3</v>
-      </c>
-      <c r="J7">
-        <v>60</v>
-      </c>
-      <c r="K7">
-        <v>0.01</v>
-      </c>
-      <c r="L7">
-        <v>30</v>
-      </c>
-      <c r="M7">
-        <v>0.01</v>
-      </c>
-      <c r="N7">
-        <v>6</v>
-      </c>
-      <c r="O7">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>12</v>
-      </c>
-      <c r="F8">
-        <v>4</v>
-      </c>
-      <c r="G8">
-        <v>11</v>
-      </c>
-      <c r="H8">
-        <v>10</v>
-      </c>
-      <c r="I8">
-        <v>5</v>
-      </c>
-      <c r="J8">
-        <v>60</v>
-      </c>
-      <c r="K8">
-        <v>0.01</v>
-      </c>
-      <c r="L8">
-        <v>30</v>
-      </c>
       <c r="M8">
-        <v>0.01</v>
-      </c>
-      <c r="N8">
-        <v>6</v>
-      </c>
-      <c r="O8">
         <v>25</v>
       </c>
     </row>

</xml_diff>